<commit_message>
chore: update midweek data workbook
</commit_message>
<xml_diff>
--- a/Midweek_Data.xlsx
+++ b/Midweek_Data.xlsx
@@ -799,21 +799,21 @@
         <v>3</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>7589</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>0/3</t>
+          <t>3/3</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I3" t="inlineStr"/>
     </row>
@@ -832,21 +832,21 @@
         <v>3</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>470</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>0/3</t>
+          <t>3/3</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I4" t="inlineStr"/>
     </row>
@@ -865,21 +865,21 @@
         <v>3</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>0/3</t>
+          <t>2/3</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I5" t="inlineStr"/>
     </row>
@@ -898,21 +898,21 @@
         <v>2</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>0/2</t>
+          <t>2/2</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I6" t="inlineStr"/>
     </row>
@@ -931,21 +931,21 @@
         <v>2</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>106</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>0/2</t>
+          <t>2/2</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I7" t="inlineStr"/>
     </row>
@@ -964,21 +964,21 @@
         <v>2</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>0/2</t>
+          <t>2/2</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I8" t="inlineStr"/>
     </row>
@@ -997,21 +997,21 @@
         <v>2</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>0/2</t>
+          <t>2/2</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I9" t="inlineStr"/>
     </row>
@@ -1129,21 +1129,21 @@
         <v>4</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>1160</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>0/4</t>
+          <t>1/4</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I3" t="inlineStr"/>
     </row>
@@ -1195,21 +1195,21 @@
         <v>3</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>3700</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>0/3</t>
+          <t>2/3</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I5" t="inlineStr"/>
     </row>
@@ -1261,21 +1261,21 @@
         <v>4</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>81</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>0/4</t>
+          <t>1/4</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I7" t="inlineStr"/>
     </row>
@@ -1294,21 +1294,21 @@
         <v>3</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>0/3</t>
+          <t>1/3</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I8" t="inlineStr"/>
     </row>
@@ -1327,21 +1327,21 @@
         <v>7</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>168</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>0/7</t>
+          <t>3/7</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I9" t="inlineStr"/>
     </row>
@@ -1360,21 +1360,21 @@
         <v>4</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="E10" t="n">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>0/4</t>
+          <t>1/4</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I10" t="inlineStr"/>
     </row>
@@ -1393,21 +1393,21 @@
         <v>5</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>130</v>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>0/5</t>
+          <t>2/5</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I11" t="inlineStr"/>
     </row>
@@ -1426,21 +1426,21 @@
         <v>3</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>1419</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>0/3</t>
+          <t>2/3</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I12" t="inlineStr"/>
     </row>
@@ -1459,23 +1459,27 @@
         <v>3</v>
       </c>
       <c r="D13" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E13" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>0/3</t>
+          <t>2/3</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>3</v>
-      </c>
-      <c r="I13" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Bacenta Sum</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1624,23 +1628,27 @@
         <v>4</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>0/4</t>
+          <t>2/4</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>4</v>
-      </c>
-      <c r="I4" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Bacenta Sum</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1921,21 +1929,21 @@
         <v>3</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>0/3</t>
+          <t>2/3</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I3" t="inlineStr"/>
     </row>
@@ -1987,21 +1995,21 @@
         <v>2</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>0/2</t>
+          <t>1/2</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I5" t="inlineStr"/>
     </row>
@@ -2020,21 +2028,21 @@
         <v>2</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>371</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>0/2</t>
+          <t>2/2</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I6" t="inlineStr"/>
     </row>
@@ -2053,21 +2061,21 @@
         <v>4</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>0/4</t>
+          <t>1/4</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I7" t="inlineStr"/>
     </row>
@@ -2086,21 +2094,21 @@
         <v>1</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>0/1</t>
+          <t>1/1</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I8" t="inlineStr"/>
     </row>
@@ -2218,21 +2226,21 @@
         <v>3</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>385</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>0/3</t>
+          <t>2/3</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I3" t="inlineStr"/>
     </row>
@@ -2251,23 +2259,27 @@
         <v>2</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>628</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>0/2</t>
+          <t>1/2</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>2</v>
-      </c>
-      <c r="I4" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Bacenta Sum</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2383,21 +2395,21 @@
         <v>3</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>0/3</t>
+          <t>3/3</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I3" t="inlineStr"/>
     </row>
@@ -2416,21 +2428,21 @@
         <v>3</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>0/3</t>
+          <t>3/3</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I4" t="inlineStr"/>
     </row>
@@ -2449,21 +2461,21 @@
         <v>6</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>0/6</t>
+          <t>6/6</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="I5" t="inlineStr"/>
     </row>
@@ -2482,23 +2494,27 @@
         <v>4</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>140</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>0/4</t>
+          <t>4/4</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>4</v>
-      </c>
-      <c r="I6" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Bacenta Sum</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2515,21 +2531,21 @@
         <v>5</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>0/5</t>
+          <t>3/5</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I7" t="inlineStr"/>
     </row>
@@ -2548,21 +2564,21 @@
         <v>5</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>185</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>0/5</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I8" t="inlineStr"/>
     </row>
@@ -2581,21 +2597,21 @@
         <v>3</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>0/3</t>
+          <t>3/3</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I9" t="inlineStr"/>
     </row>
@@ -2614,21 +2630,21 @@
         <v>3</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>0/3</t>
+          <t>2/3</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I10" t="inlineStr"/>
     </row>
@@ -2647,21 +2663,21 @@
         <v>3</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>166</v>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>0/3</t>
+          <t>3/3</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I11" t="inlineStr"/>
     </row>
@@ -2779,21 +2795,21 @@
         <v>6</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>0/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I3" t="inlineStr"/>
     </row>
@@ -2845,21 +2861,21 @@
         <v>4</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>73</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>0/4</t>
+          <t>2/4</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I5" t="inlineStr"/>
     </row>
@@ -2878,21 +2894,21 @@
         <v>5</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>358</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>0/5</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="I6" t="inlineStr"/>
     </row>
@@ -3010,21 +3026,21 @@
         <v>5</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>127</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>0/5</t>
+          <t>3/5</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I3" t="inlineStr"/>
     </row>
@@ -3043,21 +3059,21 @@
         <v>3</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>0/3</t>
+          <t>2/3</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I4" t="inlineStr"/>
     </row>
@@ -3076,21 +3092,21 @@
         <v>8</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>185</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>0/8</t>
+          <t>8/8</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="I5" t="inlineStr"/>
     </row>
@@ -3142,21 +3158,21 @@
         <v>2</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>0/2</t>
+          <t>2/2</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I7" t="inlineStr"/>
     </row>
@@ -3175,21 +3191,21 @@
         <v>3</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>1145</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>0/3</t>
+          <t>2/3</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I8" t="inlineStr"/>
     </row>
@@ -3208,21 +3224,21 @@
         <v>6</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>580</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>0/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I9" t="inlineStr"/>
     </row>
@@ -3241,21 +3257,21 @@
         <v>3</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E10" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>0/3</t>
+          <t>2/3</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I10" t="inlineStr"/>
     </row>
@@ -3274,21 +3290,21 @@
         <v>4</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>0/4</t>
+          <t>3/4</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I11" t="inlineStr"/>
     </row>
@@ -3307,21 +3323,21 @@
         <v>5</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>948</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>0/5</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I12" t="inlineStr"/>
     </row>
@@ -3340,21 +3356,21 @@
         <v>9</v>
       </c>
       <c r="D13" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>0</v>
+        <v>115</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>0/9</t>
+          <t>5/9</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="I13" t="inlineStr"/>
     </row>
@@ -3472,21 +3488,21 @@
         <v>5</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>520</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>0/5</t>
+          <t>1/5</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I3" t="inlineStr"/>
     </row>
@@ -3505,23 +3521,27 @@
         <v>3</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>172</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>0/3</t>
+          <t>3/3</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>3</v>
-      </c>
-      <c r="I4" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Bacenta Sum</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3538,21 +3558,21 @@
         <v>4</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>0/4</t>
+          <t>2/4</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I5" t="inlineStr"/>
     </row>
@@ -3571,21 +3591,21 @@
         <v>3</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>135</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>0/3</t>
+          <t>1/3</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I6" t="inlineStr"/>
     </row>
@@ -3604,21 +3624,21 @@
         <v>2</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>0/2</t>
+          <t>2/2</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I7" t="inlineStr"/>
     </row>
@@ -3637,21 +3657,21 @@
         <v>6</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>195</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>0/6</t>
+          <t>6/6</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="I8" t="inlineStr"/>
     </row>
@@ -3670,23 +3690,27 @@
         <v>1</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>0/1</t>
+          <t>1/1</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>1</v>
-      </c>
-      <c r="I9" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Bacenta Sum</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">

</xml_diff>